<commit_message>
fix: validate tabular BOM quantities
</commit_message>
<xml_diff>
--- a/fixtures/bom/fields.xlsx
+++ b/fixtures/bom/fields.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empty" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,6 +414,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>